<commit_message>
fix: preserva posicoes das colunas no cadastro
</commit_message>
<xml_diff>
--- a/docs/CadastroCoroinhas.xlsx
+++ b/docs/CadastroCoroinhas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\EscalaCoroinhas\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3ACC117-20BB-4B5B-8217-34E224AA6E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6005A267-3EBE-4416-B258-833ECC08EFA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{C1CD5EC7-63F8-4159-BB4E-CAD1935FD014}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="57">
   <si>
     <t>Coroinhas</t>
   </si>
@@ -207,6 +208,9 @@
   </si>
   <si>
     <t>td</t>
+  </si>
+  <si>
+    <t>Experiências</t>
   </si>
 </sst>
 </file>
@@ -279,16 +283,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C2E4232-FC25-4BD5-9B83-1038F48F2D80}" name="coroinhas" displayName="coroinhas" ref="A1:D48" totalsRowShown="0">
-  <autoFilter ref="A1:D48" xr:uid="{2C2E4232-FC25-4BD5-9B83-1038F48F2D80}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C2E4232-FC25-4BD5-9B83-1038F48F2D80}" name="coroinhas" displayName="coroinhas" ref="A1:E48" totalsRowShown="0">
+  <autoFilter ref="A1:E48" xr:uid="{2C2E4232-FC25-4BD5-9B83-1038F48F2D80}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C48">
     <sortCondition ref="C1:C48"/>
   </sortState>
-  <tableColumns count="4">
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{9E736BA1-00B8-461F-8EB2-79EE6D8CAB80}" name="Coroinhas"/>
     <tableColumn id="2" xr3:uid="{9C3A8BF2-A130-4D84-BBDE-4E0387D0C719}" name="data nascimento" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{FDE52173-27E7-4DDA-86BC-02F21E0A69A4}" name="função"/>
     <tableColumn id="4" xr3:uid="{28E5B8D5-028C-4B06-86E7-384268309D96}" name="Horario"/>
+    <tableColumn id="5" xr3:uid="{86B155D8-C10C-45B2-8A2A-28B479788F0E}" name="Experiências"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -611,16 +616,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E2DE50D-91EA-4031-83F4-7BFDD3AA51B8}">
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" style="1" customWidth="1"/>
     <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -633,8 +639,11 @@
       <c r="D1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -647,8 +656,11 @@
       <c r="D2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -661,8 +673,11 @@
       <c r="D3" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -675,8 +690,11 @@
       <c r="D4" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -689,8 +707,11 @@
       <c r="D5" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -703,8 +724,11 @@
       <c r="D6" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -717,8 +741,11 @@
       <c r="D7" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -731,8 +758,11 @@
       <c r="D8" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -745,8 +775,11 @@
       <c r="D9" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>45</v>
       </c>
@@ -759,8 +792,11 @@
       <c r="D10" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>48</v>
       </c>
@@ -773,8 +809,11 @@
       <c r="D11" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>50</v>
       </c>
@@ -787,8 +826,11 @@
       <c r="D12" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>52</v>
       </c>
@@ -801,8 +843,11 @@
       <c r="D13" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -815,8 +860,11 @@
       <c r="D14" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -827,10 +875,13 @@
         <v>4</v>
       </c>
       <c r="D15" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -843,8 +894,11 @@
       <c r="D16" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -857,8 +911,11 @@
       <c r="D17" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>46</v>
       </c>
@@ -871,8 +928,11 @@
       <c r="D18" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>5</v>
       </c>
@@ -885,8 +945,11 @@
       <c r="D19" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>7</v>
       </c>
@@ -899,8 +962,11 @@
       <c r="D20" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -913,8 +979,11 @@
       <c r="D21" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -927,8 +996,11 @@
       <c r="D22" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -941,8 +1013,11 @@
       <c r="D23" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>14</v>
       </c>
@@ -955,8 +1030,11 @@
       <c r="D24" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>18</v>
       </c>
@@ -969,8 +1047,11 @@
       <c r="D25" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>20</v>
       </c>
@@ -983,8 +1064,11 @@
       <c r="D26" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -995,10 +1079,13 @@
         <v>6</v>
       </c>
       <c r="D27" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="E27">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -1011,8 +1098,11 @@
       <c r="D28" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>24</v>
       </c>
@@ -1025,8 +1115,11 @@
       <c r="D29" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>25</v>
       </c>
@@ -1039,8 +1132,11 @@
       <c r="D30" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>26</v>
       </c>
@@ -1053,8 +1149,11 @@
       <c r="D31" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>27</v>
       </c>
@@ -1067,8 +1166,11 @@
       <c r="D32" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>30</v>
       </c>
@@ -1081,8 +1183,11 @@
       <c r="D33" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>31</v>
       </c>
@@ -1095,8 +1200,11 @@
       <c r="D34" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>33</v>
       </c>
@@ -1109,8 +1217,11 @@
       <c r="D35" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -1123,8 +1234,11 @@
       <c r="D36" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -1137,8 +1251,11 @@
       <c r="D37" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>37</v>
       </c>
@@ -1151,8 +1268,11 @@
       <c r="D38" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -1165,8 +1285,11 @@
       <c r="D39" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -1179,8 +1302,11 @@
       <c r="D40" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>40</v>
       </c>
@@ -1193,8 +1319,11 @@
       <c r="D41" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>41</v>
       </c>
@@ -1207,8 +1336,11 @@
       <c r="D42" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>42</v>
       </c>
@@ -1221,8 +1353,11 @@
       <c r="D43" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>43</v>
       </c>
@@ -1235,8 +1370,11 @@
       <c r="D44" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>44</v>
       </c>
@@ -1249,8 +1387,11 @@
       <c r="D45" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E45">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>47</v>
       </c>
@@ -1263,8 +1404,11 @@
       <c r="D46" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>49</v>
       </c>
@@ -1277,8 +1421,11 @@
       <c r="D47" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>51</v>
       </c>
@@ -1290,6 +1437,9 @@
       </c>
       <c r="D48" t="s">
         <v>55</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>